<commit_message>
update main page product data grid view
</commit_message>
<xml_diff>
--- a/src/data/products-data.xlsx
+++ b/src/data/products-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyanc\VScodeProgram\inteplast_home_page_tw\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20725A43-4ED5-4F1E-BCA9-7A707DE1D4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5C559F2-6D22-45FF-B57E-E9B04B930074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -100,10 +100,6 @@
     <t>Can Liners</t>
   </si>
   <si>
-    <t>一拉即束口，防止臭味外溢。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>集團專利抽取式秤紙。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -129,6 +125,32 @@
   </si>
   <si>
     <t>專利證書</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>一拉即束口</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Microsoft JhengHei UI"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>，多30%以上使用容量</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="新細明體"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>，並可防止臭味外溢。</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -136,7 +158,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -150,6 +172,13 @@
       <family val="3"/>
       <charset val="136"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Microsoft JhengHei UI"/>
+      <family val="2"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="2">
@@ -548,13 +577,13 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
         <v>17</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -568,7 +597,7 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -579,13 +608,13 @@
         <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -596,13 +625,13 @@
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -630,7 +659,7 @@
         <v>16</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
update product information - add notice line
</commit_message>
<xml_diff>
--- a/src/data/products-data.xlsx
+++ b/src/data/products-data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyanc\VScodeProgram\inteplast_home_page_tw\src\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyanc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975C0869-C802-46F5-9353-B786DB90E1E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413DDD4D-F556-4EB5-A2B6-868A32C835E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>產品</t>
   </si>
@@ -33,6 +33,9 @@
     <t>英文名稱</t>
   </si>
   <si>
+    <t>重點</t>
+  </si>
+  <si>
     <t>產品敘述</t>
   </si>
   <si>
@@ -57,9 +60,6 @@
     <t>蔬果袋</t>
   </si>
   <si>
-    <t>食品級原料，平裝、捲裝耐熱袋與蔬果袋。</t>
-  </si>
-  <si>
     <t>封面-蔬果袋.png</t>
   </si>
   <si>
@@ -69,132 +69,153 @@
     <t>多功能手套</t>
   </si>
   <si>
-    <t/>
+    <t>封面-Scale Sheet.png</t>
+  </si>
+  <si>
+    <t>專利證書</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Produce Bag</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>耐熱袋、雙道封口、食品袋、市場袋</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Can Liners</t>
+  </si>
+  <si>
+    <t>連捲、單張抽取、八折袋、環保清潔袋</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Draw Tape Liners</t>
+  </si>
+  <si>
+    <t>清潔袋、醫療袋、環保拉繩袋</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Multifunctional Gloves</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>封面-多功能手套.png</t>
+  </si>
+  <si>
+    <t>無粉末、無乳膠、內壓紋、易穿脫、彈性優、觸感佳</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Recloseable Zipper Bags</t>
+  </si>
+  <si>
+    <t>封面-夾鏈袋.png</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>密實袋、冷凍袋、夾鏈袋</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>遮蔽防塵膠帶</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pre-Taped Masking Film</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>封面-台塑遮蔽防塵膠帶.png</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>遮蔽保護、消毒防護、覆蓋防塵、施工便利</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>Scale Sheet</t>
-  </si>
-  <si>
-    <t>封面-夾鏈袋.png</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>封面-多功能手套.png</t>
-  </si>
-  <si>
-    <t>遮蔽防塵膠帶</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>封面-台塑遮蔽防塵膠帶.png</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Draw Tape Liners</t>
-  </si>
-  <si>
-    <t>Can Liners</t>
-  </si>
-  <si>
-    <t>集團專利抽取式秤紙。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>連捲、單張抽取與環保清潔袋。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>密實袋、冷凍袋、夾鏈袋</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>清潔袋、醫療袋、環保拉繩袋</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>專利證書</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>封面-Scale Sheet.png</t>
-  </si>
-  <si>
-    <t>Produce Bag</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>連捲、單張抽取、八折袋、環保清潔袋</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Multifunctional Gloves</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>內壓紋、易穿脫、彈性優、觸感佳</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>無粉末、無乳膠</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>一拉即束口，多30%以上使用容量，並可防止臭味外溢。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Recloseable Zipper Bags</t>
-  </si>
-  <si>
-    <t>遮蔽保護、消毒防護、覆蓋防塵、施工便利</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>手感扎實、夾鏈緊密、多次使用</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Pre-Taped Masking Film</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>耐熱袋</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Microsoft JhengHei UI"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>、雙道封口</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="微軟正黑體"/>
-        <family val="2"/>
-        <charset val="136"/>
-      </rPr>
-      <t>、食品袋、市場袋</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>一拉即束口，容量大升級增加 30% 、乾淨不沾手</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>專為現代便利生活與高效清潔設計的貼心之作。一體成型的堅固拉繩結構，讓您輕鬆一拉即可俐落束口，有效避免清理時垃圾外漏與雙手沾染髒汙的困擾。特殊設計使內部空間有效利用率增加 30% 以上，並能緊密鎖住異味不外散；另提供醫療級與環保拉繩款式，讓居家與商辦環境更顯潔淨衛生。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>兼具極佳彈性與細緻觸感的多功能手套系列。表面採特殊內壓紋設計，不僅穿脫滑順、不沾黏，更具備良好的防滑抓握力。全系列符合無粉末、無乳膠等友善肌膚標準，無論是用於餐飲調理、食品加工、日常清潔打掃或居家照護，皆能提供全方位且靈活舒適的衛生防護體驗。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>親膚舒適、防護俐落的萬用防護手套</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">
+結合集團專利技術打造的抽取式 Scale Sheet，打破傳統取用的繁瑣與不便。採用貼心的單張抽取設計，不僅取用俐落、大幅節省作業時間，更能有效管控使用成本。質地強韌、防沾黏且不易破損，是生鮮秤重、餐飲備料、工業分裝及各大商場櫃台追求高效率作業的不可或缺的專業首選。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tare Sheet，集團專利抽取式設計，極致提升效率</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>強韌耐穿刺、滴水不漏的日常清潔首選</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>依託台塑高品質原料自製優勢，經由嘉義新港廠區自動化精密吹膜與封口技術打造。全系列涵蓋連捲式、單張抽取式及國家環保標章認證清潔袋等多種款式。具備超強的抗拉張力與優異承重力，不論是用於一般家庭日常垃圾清運，或是辦公大樓、餐飲旅宿等高頻率商用場域，皆能輕鬆應對、安心不破漏。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>食品級安心原料，守護食材新鮮與衛生</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>專為生鮮食品與日常零售打造的優質蔬果袋系列。嚴選食品級合格原料，質地安全、無毒無味，具備極佳的透明度與抗拉韌性。提供平裝、捲裝等多樣化規格，搭配耐熱袋、雙道封口食品袋及市場專用袋等多元選擇，有效鎖住食材水分與鮮度，為消費者與商家嚴格把關每一道飲食安全防線。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">
+採用高標準工藝打造的重覆使用夾鏈袋系列。袋身厚實、手感紮實，搭配密合度極佳的雙軌或單軌夾鏈結構，具備優異的氣密與防潮表現。不論是生鮮食材冷凍保鮮、日常小物分類收納，或是工業零件包裝，皆能提供卓越的密封保護，支援多次重複開合依然緊密如初。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>手感紮實、密封緊密，完美鎖住鮮度與整潔</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">
+集膠帶與防塵膜於一體的便利防護方案。專為室內裝潢、噴漆粉刷、居家裝修及醫療消毒防護設計，能夠快速且大面積地覆蓋並保護傢俱、地板與牆面免受粉塵、油漆噴濺汙染。黏貼穩固且撕除不留殘膠，大幅簡化施工前的遮蔽前置作業，兼具高效率與完美防護效果。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>施工裝潢與日常防塵的省時利器</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="新細明體"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Noto Serif HK Medium"/>
+      <family val="1"/>
+      <charset val="136"/>
     </font>
     <font>
       <sz val="9"/>
@@ -206,21 +227,8 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="微軟正黑體"/>
-      <family val="2"/>
-      <charset val="136"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF3C535D"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Microsoft JhengHei UI"/>
-      <family val="2"/>
+      <name val="Noto Serif HK Medium"/>
+      <family val="1"/>
       <charset val="136"/>
     </font>
   </fonts>
@@ -244,14 +252,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -592,158 +606,191 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="30.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="61.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="16.21875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.44140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="88" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="33" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="59.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="46.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" ht="19.8" x14ac:dyDescent="0.5">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="99" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="79.2" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>38</v>
-      </c>
+      <c r="F3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="79.2" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>29</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="79.2" x14ac:dyDescent="0.5">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>8</v>
+      <c r="D5" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>25</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="79.2" x14ac:dyDescent="0.5">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>17</v>
+      <c r="B6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>32</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="3"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="99" x14ac:dyDescent="0.5">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>16</v>
+      <c r="B7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>43</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>24</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="99" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>19</v>
+        <v>29</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>45</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="3"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E1 A6 A5 A4 D4 D5" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:F1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update Scale sheet 產品名稱敘述更正
</commit_message>
<xml_diff>
--- a/src/data/products-data.xlsx
+++ b/src/data/products-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lyanc\VScodeProgram\inteplast_home_page_tw\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51D752CB-EF9D-4A90-800A-0778F44FE35A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07C97469-AD6C-4A19-9645-FDAA6C8A871C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -93,9 +93,6 @@
     <t>清潔袋</t>
   </si>
   <si>
-    <t>Can Liners</t>
-  </si>
-  <si>
     <t>強韌耐穿刺、滴水不漏的日常清潔首選</t>
   </si>
   <si>
@@ -114,9 +111,6 @@
     <t>連捲、單張抽取、八折袋、環保清潔袋</t>
   </si>
   <si>
-    <t>Perforated roll, Single-sheet dispensing, Eight-fold gusseted bag, Green Mark liner</t>
-  </si>
-  <si>
     <t>拉繩袋</t>
   </si>
   <si>
@@ -225,20 +219,29 @@
     <t>Masking protection, Disinfection screening, Dust cover, Fast application</t>
   </si>
   <si>
-    <t>Scale Sheet(Tare Sheet)</t>
+    <t>結合集團專利技術打造的抽取式 Scale Sheet，突破傳統取用方式的繁瑣與不便。採用貼心的單張抽取設計，取用俐落、操作便利，不僅能提升作業效率、節省取用時間，更能有效控管使用成本。材質強韌、防沾黏且不易受污染，適用於生鮮秤重、餐飲備料、工業分裝及各大商場櫃台等多元作業場景，是追求高效率、衛生與便利性的專業首選。</t>
+  </si>
+  <si>
+    <t>Featuring the Group’s patented pull-out technology, Scale Sheet offers a smarter and more convenient alternative to traditional dispensing methods. Its easy-to-use single-sheet dispensing design allows for quick and efficient access, helping save valuable operation time while providing better control over material usage and costs. Durable, non-stick, and resistant to contamination, Scale Sheet is ideal for fresh food weighing, food preparation, industrial packaging, and retail counter operations, making it a professional choice for businesses seeking greater efficiency, hygiene, and convenience.</t>
+  </si>
+  <si>
+    <t>集團專利單張抽取設計｜取用便利・不易污染・衛生安心</t>
+  </si>
+  <si>
+    <t>Patented Single-Sheet Dispensing | Easy to Use, Reduced Contamination, Improved Hygiene</t>
+  </si>
+  <si>
+    <t>Garbage Bag</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>結合集團專利技術打造的抽取式 Scale Sheet，突破傳統取用方式的繁瑣與不便。採用貼心的單張抽取設計，取用俐落、操作便利，不僅能提升作業效率、節省取用時間，更能有效控管使用成本。材質強韌、防沾黏且不易受污染，適用於生鮮秤重、餐飲備料、工業分裝及各大商場櫃台等多元作業場景，是追求高效率、衛生與便利性的專業首選。</t>
-  </si>
-  <si>
-    <t>Featuring the Group’s patented pull-out technology, Scale Sheet offers a smarter and more convenient alternative to traditional dispensing methods. Its easy-to-use single-sheet dispensing design allows for quick and efficient access, helping save valuable operation time while providing better control over material usage and costs. Durable, non-stick, and resistant to contamination, Scale Sheet is ideal for fresh food weighing, food preparation, industrial packaging, and retail counter operations, making it a professional choice for businesses seeking greater efficiency, hygiene, and convenience.</t>
-  </si>
-  <si>
-    <t>集團專利單張抽取設計｜取用便利・不易污染・衛生安心</t>
-  </si>
-  <si>
-    <t>Patented Single-Sheet Dispensing | Easy to Use, Reduced Contamination, Improved Hygiene</t>
+    <t>Perforated roll, Single-sheet dispensing, Can Liners, ECO Garbage Bag</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scale Sheet
+(Tare Sheet)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -686,22 +689,22 @@
     </row>
     <row r="2" spans="1:9" s="2" customFormat="1" ht="97.2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>9</v>
@@ -747,144 +750,144 @@
         <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="E4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="I4" s="1" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:9" s="2" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="I5" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:9" s="2" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:9" s="2" customFormat="1" ht="62.4" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="G7" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:9" s="2" customFormat="1" ht="78" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -892,7 +895,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I1 A3:I8 G2:I2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I1 A3:I3 G2:I2 A5:I8 A4 C4:H4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>